<commit_message>
have a nice day
</commit_message>
<xml_diff>
--- a/uploads/ORIGINAL7.xlsx
+++ b/uploads/ORIGINAL7.xlsx
@@ -25270,8 +25270,8 @@
       <c r="L20" s="226" t="s">
         <v>47</v>
       </c>
-      <c r="M20" s="205" t="s">
-        <v>49</v>
+      <c r="M20" s="57" t="s">
+        <v>48</v>
       </c>
       <c r="N20" s="206" t="s">
         <v>46</v>
@@ -25291,8 +25291,8 @@
       <c r="S20" s="214" t="s">
         <v>46</v>
       </c>
-      <c r="T20" s="205" t="s">
-        <v>49</v>
+      <c r="T20" s="57" t="s">
+        <v>48</v>
       </c>
       <c r="U20" s="206" t="s">
         <v>45</v>
@@ -25357,11 +25357,11 @@
       </c>
       <c r="AN20" s="52">
         <f t="shared" ref="AN20:AO20" si="22">COUNTIF($C20:$AF20,"PH")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AO20" s="52">
         <f t="shared" si="22"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AP20" s="67"/>
       <c r="AQ20" s="67"/>
@@ -30062,7 +30062,7 @@
       </c>
       <c r="M56" s="275">
         <f t="shared" si="59"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N56" s="140">
         <f t="shared" si="59"/>
@@ -30090,7 +30090,7 @@
       </c>
       <c r="T56" s="275">
         <f t="shared" si="59"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U56" s="140">
         <f t="shared" si="59"/>
@@ -30202,7 +30202,7 @@
       </c>
       <c r="M57" s="275">
         <f t="shared" si="60"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N57" s="140">
         <f t="shared" si="60"/>
@@ -30230,7 +30230,7 @@
       </c>
       <c r="T57" s="275">
         <f t="shared" si="60"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U57" s="140">
         <f t="shared" si="60"/>
@@ -42562,7 +42562,7 @@
         <v>47</v>
       </c>
       <c r="M18" s="288" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N18" s="288" t="s">
         <v>46</v>
@@ -42583,7 +42583,7 @@
         <v>46</v>
       </c>
       <c r="T18" s="288" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="U18" s="288" t="s">
         <v>45</v>
@@ -47792,7 +47792,7 @@
         <v>4.0</v>
       </c>
       <c r="L9" s="298">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="M9" s="287">
         <v>0.0</v>
@@ -47813,7 +47813,7 @@
         <v>2.0</v>
       </c>
       <c r="S9" s="298">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="T9" s="287">
         <v>0.0</v>
@@ -47887,7 +47887,7 @@
         <v>2.0</v>
       </c>
       <c r="L10" s="298">
-        <v>5.0</v>
+        <v>4.0</v>
       </c>
       <c r="M10" s="287">
         <v>4.0</v>
@@ -47908,7 +47908,7 @@
         <v>3.0</v>
       </c>
       <c r="S10" s="298">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="T10" s="287">
         <v>5.0</v>
@@ -51789,7 +51789,7 @@
         <v>47</v>
       </c>
       <c r="M18" s="288" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N18" s="288" t="s">
         <v>46</v>
@@ -51810,7 +51810,7 @@
         <v>46</v>
       </c>
       <c r="T18" s="288" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="U18" s="288" t="s">
         <v>45</v>

</xml_diff>